<commit_message>
Push all current local changes
</commit_message>
<xml_diff>
--- a/uploads/GK2400128-_SOB.xlsx
+++ b/uploads/GK2400128-_SOB.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://manomayconsultancyservices-my.sharepoint.com/personal/guruprasad_mekala_manomay_biz/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://manomayconsultancyservices-my.sharepoint.com/personal/guruprasad_mekala_manomay_biz/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{51EA5990-CDC2-4CD6-9D3E-8578640D965E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE2525E3-ED37-4FBD-8CC8-647D128EC867}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACBFCBED-53E8-4BD6-AD22-E40D3C1A2AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{652612B8-CFC8-4FA2-81CD-6EFACED5E565}"/>
   </bookViews>

</xml_diff>